<commit_message>
Table S1 actions: Institutions x R4.2 per the corrected supplement
The cell duplicated Institutions x R1.2 (licensing/consent, data
stewardship); the corrected Table S1 has two cost-benefit actions there.
Both workbooks updated identically; page re-rendered.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_publication_static/TIER2_recommendations.xlsx
+++ b/01_publication_static/TIER2_recommendations.xlsx
@@ -2235,7 +2235,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Clarify licensing, consent and data-protection conditions for data held or generated at the institution, so that secondary users know what re-use is permitted</t>
+          <t>Track the staff time and costs of institutional reproducibility measures, such as training, support roles and data stewardship, and make these data available to meta-researchers under appropriate access conditions</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Provide data stewardship and legal support to help researchers assess whether and how existing data may be re-used</t>
+          <t>Evaluate the costs and benefits of own training and policy programmes, including unintended effects on researchers' workload, and publish the results</t>
         </is>
       </c>
     </row>

</xml_diff>